<commit_message>
Updated files until today
</commit_message>
<xml_diff>
--- a/3. MusicAndArts/1. CarnaticMusicPlusOthers/0. Books/SahajayogaBhajansAndNotes/0. Bhajans_WithWordToWordTranslations/3.3. HW-14112025-Music-Song-Breakdown-Mata-Nirmala-Maheshvari.xlsx
+++ b/3. MusicAndArts/1. CarnaticMusicPlusOthers/0. Books/SahajayogaBhajansAndNotes/0. Bhajans_WithWordToWordTranslations/3.3. HW-14112025-Music-Song-Breakdown-Mata-Nirmala-Maheshvari.xlsx
@@ -9,10 +9,33 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="e/Y96SeDxFSPPwV5UoRaqyXPCZTLEAQnDqEC9wQ0wx4="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="KOZ01V4qXnFzlndw2gc/86fGxoxvhmnYz2KFAVwcyCk="/>
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment authorId="0" ref="B71">
+      <text>
+        <t xml:space="preserve">======
+ID#AAAB1_sajM4
+Virata Pusuluri    (2026-03-17 18:27:38)
+Ni Ni Nii Ni Ma Maa should be replaced with Sa+ Sa+ Sa+: Sa+ Ma Maa</t>
+      </text>
+    </comment>
+  </commentList>
+  <extLst>
+    <ext uri="GoogleSheetsCustomDataVersion2">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7miO5f8rj1wVGaxcC9qu9xCHsWMoRg=="/>
+    </ext>
+  </extLst>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17895,6 +17918,7 @@
     <mergeCell ref="E55:G55"/>
     <mergeCell ref="H55:K55"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>